<commit_message>
updates houston-common and simple testplans
</commit_message>
<xml_diff>
--- a/docs/test-plans/45drives-storage-wizard-simple-test-plan-linux.xlsx
+++ b/docs/test-plans/45drives-storage-wizard-simple-test-plan-linux.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Plan'!$A$1:$J$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Plan'!$A$1:$J$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10">
@@ -596,6 +596,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr"/>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
@@ -625,7 +626,7 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
@@ -665,7 +666,7 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22">
@@ -685,7 +686,7 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24">
@@ -695,7 +696,7 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -709,7 +710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J57"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -787,7 +788,7 @@
           <t>1.1</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr"/>
+      <c r="C2" s="4" t="n"/>
       <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Install the app</t>
@@ -805,10 +806,10 @@
           <t>The app installs with no error messages, it appears in your applications menu, and clicking it opens the app.</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr"/>
-      <c r="H2" s="4" t="inlineStr"/>
-      <c r="I2" s="4" t="inlineStr"/>
-      <c r="J2" s="4" t="inlineStr"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
+      <c r="I2" s="4" t="n"/>
+      <c r="J2" s="4" t="n"/>
     </row>
     <row r="3" ht="49.5" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -821,7 +822,7 @@
           <t>1.2</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="n"/>
       <c r="D3" s="5" t="inlineStr">
         <is>
           <t>The app opens to the Dashboard</t>
@@ -837,12 +838,12 @@
           <t>You see a page called Dashboard. Nothing is blank, nothing is spinning forever, and there are no error messages.</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr"/>
-      <c r="I3" s="5" t="inlineStr"/>
-      <c r="J3" s="5" t="inlineStr"/>
-    </row>
-    <row r="4" ht="49.5" customHeight="1">
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="5" t="n"/>
+      <c r="J3" s="5" t="n"/>
+    </row>
+    <row r="4" ht="64" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>1. Install the App</t>
@@ -853,7 +854,7 @@
           <t>1.3</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="n"/>
       <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Check the app name at the top</t>
@@ -866,13 +867,13 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>It says 45Drives Storage Wizard and a version number, for example v1.4.0. Write the version number in the Notes column.</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr"/>
-      <c r="I4" s="5" t="inlineStr"/>
-      <c r="J4" s="5" t="inlineStr"/>
+          <t>It says 45Drives Storage Wizard and a version number, for example v1.6.4. Write the version number in the Notes column.</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n"/>
+      <c r="I4" s="5" t="n"/>
+      <c r="J4" s="5" t="n"/>
     </row>
     <row r="5" ht="49.5" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -885,7 +886,7 @@
           <t>2.1</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr"/>
+      <c r="C5" s="4" t="n"/>
       <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Find the Quick Actions buttons</t>
@@ -903,12 +904,12 @@
           <t>You see five buttons: Setup Single Server, Setup Multiple Servers, Manage Backups, Logs, and Settings.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr"/>
-      <c r="I5" s="4" t="inlineStr"/>
-      <c r="J5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6" ht="49.5" customHeight="1">
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="n"/>
+    </row>
+    <row r="6" ht="93" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>2. Look Around the App</t>
@@ -919,46 +920,80 @@
           <t>2.2</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="n"/>
       <c r="D6" s="5" t="inlineStr">
         <is>
+          <t>A guided tour shows you around</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>1. Look at the Dashboard the first time you open the app.
+2. If a box appears highlighting part of the screen, read it and click through to the end, or click Skip.
+3. Use the menu to go to another screen, then come back to the Dashboard.</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>A short guided tour appears the first time only. Once you have finished it or skipped it, it does not come back every time you return to the Dashboard.</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="5" t="n"/>
+      <c r="J6" s="5" t="n"/>
+    </row>
+    <row r="7" ht="49.5" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>2. Look Around the App</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
           <t>Open the menu</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>1. Look at the top-right corner of the app.
 2. Click the button with three flat lines on it.</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>A panel slides out from the side. It says Menu at the top, and has a Navigation list and an Appearance section.</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr"/>
-      <c r="I6" s="5" t="inlineStr"/>
-      <c r="J6" s="5" t="inlineStr"/>
-    </row>
-    <row r="7" ht="78.5" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n"/>
+      <c r="I7" s="5" t="n"/>
+      <c r="J7" s="5" t="n"/>
+    </row>
+    <row r="8" ht="78.5" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>2. Look Around the App</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>2.3</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Every menu item opens something</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>1. In the menu, click Dashboard.
 2. Open the menu again and click Setup Wizard.
@@ -967,100 +1002,100 @@
 5. Open the menu again and click Settings.</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Every single one opens a page or a box. Nothing does nothing, and nothing shows an error.</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr"/>
-      <c r="I7" s="5" t="inlineStr"/>
-      <c r="J7" s="5" t="inlineStr"/>
-    </row>
-    <row r="8" ht="35" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="5" t="n"/>
+      <c r="J8" s="5" t="n"/>
+    </row>
+    <row r="9" ht="35" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>2. Look Around the App</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>2.4</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Close the app and open it again</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>1. Close the app completely.
 2. Open it again.</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>The app opens again to the Dashboard with no errors.</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr"/>
-      <c r="H8" s="5" t="inlineStr"/>
-      <c r="I8" s="5" t="inlineStr"/>
-      <c r="J8" s="5" t="inlineStr"/>
-    </row>
-    <row r="9" ht="35" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="5" t="n"/>
+      <c r="J9" s="5" t="n"/>
+    </row>
+    <row r="10" ht="35" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>3. Set Up Your Server</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>3.1</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Start the Setup Wizard</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>1. Go back to the Dashboard.
 2. Click Setup Single Server under Quick Actions.</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>A page opens that says Welcome to the 45Drives Setup Wizard! There is a Next button at the bottom.</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr"/>
-      <c r="H9" s="4" t="inlineStr"/>
-      <c r="I9" s="4" t="inlineStr"/>
-      <c r="J9" s="4" t="inlineStr"/>
-    </row>
-    <row r="10" ht="78.5" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="n"/>
+      <c r="I10" s="4" t="n"/>
+      <c r="J10" s="4" t="n"/>
+    </row>
+    <row r="11" ht="78.5" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>3. Set Up Your Server</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr"/>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>Read the picture steps</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>1. Click Next to go to Unboxing.
 2. Click Next to go to Plug-In Power.
@@ -1069,67 +1104,67 @@
 5. Click Back once, then Next again.</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>Each step shows a picture and a short explanation. Back and Next both work. Nothing is blank or broken.</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr"/>
-      <c r="H10" s="5" t="inlineStr"/>
-      <c r="I10" s="5" t="inlineStr"/>
-      <c r="J10" s="5" t="inlineStr"/>
-    </row>
-    <row r="11" ht="35" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="G11" s="5" t="n"/>
+      <c r="H11" s="5" t="n"/>
+      <c r="I11" s="5" t="n"/>
+      <c r="J11" s="5" t="n"/>
+    </row>
+    <row r="12" ht="35" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>3. Set Up Your Server</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr"/>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Hover the question mark for help</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>1. On any step, find the small ? icon.
 2. Rest your mouse pointer on it without clicking.</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>A helpful hint appears explaining that step in plain words.</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr"/>
-      <c r="I11" s="5" t="inlineStr"/>
-      <c r="J11" s="5" t="inlineStr"/>
-    </row>
-    <row r="12" ht="93" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="G12" s="5" t="n"/>
+      <c r="H12" s="5" t="n"/>
+      <c r="I12" s="5" t="n"/>
+      <c r="J12" s="5" t="n"/>
+    </row>
+    <row r="13" ht="122" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>3. Set Up Your Server</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr"/>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Find your server in the list</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>1. Click Next until you reach the page titled Select a 45Drives Server to Setup.
 2. Click the box labelled Select a server.
@@ -1137,66 +1172,66 @@
 4. If it is not there, wait a moment and click Rescan Servers.</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>Your server appears in the list. It is shown as the server's name followed by numbers in brackets, for example MyServer (192.168.1.50).</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr"/>
-      <c r="H12" s="5" t="inlineStr"/>
-      <c r="I12" s="5" t="inlineStr"/>
-      <c r="J12" s="5" t="inlineStr"/>
-    </row>
-    <row r="13" ht="35" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>While it is looking, the box says Searching the network for servers…. When it finds something the box says — Choose a detected server — and your server is listed as its name followed by numbers in brackets, for example MyServer (192.168.1.50). If nothing is found it says No servers found — enter an IP manually. The list does not flicker or empty itself while you are looking at it.</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="n"/>
+      <c r="H13" s="5" t="n"/>
+      <c r="I13" s="5" t="n"/>
+      <c r="J13" s="5" t="n"/>
+    </row>
+    <row r="14" ht="35" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>3. Set Up Your Server</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>3.5</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr"/>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Let the app use your network</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>1. If your computer asks for permission to use the network, allow it.</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>The app keeps working. If nothing was asked, that is fine too - write 'no prompt appeared' in Notes.</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr"/>
-      <c r="H13" s="5" t="inlineStr"/>
-      <c r="I13" s="5" t="inlineStr"/>
-      <c r="J13" s="5" t="inlineStr"/>
-    </row>
-    <row r="14" ht="122" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="G14" s="5" t="n"/>
+      <c r="H14" s="5" t="n"/>
+      <c r="I14" s="5" t="n"/>
+      <c r="J14" s="5" t="n"/>
+    </row>
+    <row r="15" ht="122" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>3. Set Up Your Server</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>3.6</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr"/>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Sign in to the server</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>1. Click your server in the list to choose it.
 2. On the right, leave Username as root unless you were told otherwise.
@@ -1206,67 +1241,67 @@
 6. Click Next.</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>The wrong password gives you a clear message telling you something went wrong. The app does not freeze or close. With the right password the button changes to Installing... and after a short wait a new page appears saying Set Up Your Server.</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr"/>
-      <c r="H14" s="5" t="inlineStr"/>
-      <c r="I14" s="5" t="inlineStr"/>
-      <c r="J14" s="5" t="inlineStr"/>
-    </row>
-    <row r="15" ht="49.5" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="G15" s="5" t="n"/>
+      <c r="H15" s="5" t="n"/>
+      <c r="I15" s="5" t="n"/>
+      <c r="J15" s="5" t="n"/>
+    </row>
+    <row r="16" ht="49.5" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>3. Set Up Your Server</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>3.7</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr"/>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Choose the easy option</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>1. On the Set Up Your Server page, look at the two cards.
 2. Click the one on the left that says SIMPLE with a Recommended badge.</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>The SIMPLE card is chosen and you move to a page called Storage Server Set Up.</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr"/>
-      <c r="H15" s="5" t="inlineStr"/>
-      <c r="I15" s="5" t="inlineStr"/>
-      <c r="J15" s="5" t="inlineStr"/>
-    </row>
-    <row r="16" ht="93" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="5" t="n"/>
+      <c r="J16" s="5" t="n"/>
+    </row>
+    <row r="17" ht="93" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>3. Set Up Your Server</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>3.8</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr"/>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>The app stops you making mistakes</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>1. In Server Name, type a name with a space in it, like My Server. Look for a message.
 2. In User Name, type root. Look for a message.
@@ -1274,34 +1309,34 @@
 4. In Confirm Password, type something different to your password. Look for a message.</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>Each time, a short message in plain English tells you what is wrong, and the Next button stays greyed out until you fix it.</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr"/>
-      <c r="H16" s="5" t="inlineStr"/>
-      <c r="I16" s="5" t="inlineStr"/>
-      <c r="J16" s="5" t="inlineStr"/>
-    </row>
-    <row r="17" ht="151" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="5" t="n"/>
+      <c r="I17" s="5" t="n"/>
+      <c r="J17" s="5" t="n"/>
+    </row>
+    <row r="18" ht="151" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>3. Set Up Your Server</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>3.9</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr"/>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>Fill in your server details</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>1. In Server Name, type a simple name with no spaces, like myserver.
 2. In User Name, type a simple name in lower case, like jane.
@@ -1312,34 +1347,34 @@
 7. Look at the Folder Preview picture underneath.</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>Folder Preview shows you the address of your new folder, for example \\myserver.local\data. The Next button is no longer greyed out.</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr"/>
-      <c r="H17" s="5" t="inlineStr"/>
-      <c r="I17" s="5" t="inlineStr"/>
-      <c r="J17" s="5" t="inlineStr"/>
-    </row>
-    <row r="18" ht="78.5" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="G18" s="5" t="n"/>
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="5" t="n"/>
+      <c r="J18" s="5" t="n"/>
+    </row>
+    <row r="19" ht="78.5" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>3. Set Up Your Server</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>3.10</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr"/>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="C19" s="5" t="n"/>
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>Write your details down</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>1. Write down your Server Name, User Name, Password and Network Folder Name on paper. You cannot get them back later.
 2. Click Next.
@@ -1347,34 +1382,34 @@
 4. Click OK, Proceed.</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>A box appears warning you to save your details. Clicking OK, Proceed takes you to a page called Storage Drive Summary.</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr"/>
-      <c r="H18" s="5" t="inlineStr"/>
-      <c r="I18" s="5" t="inlineStr"/>
-      <c r="J18" s="5" t="inlineStr"/>
-    </row>
-    <row r="19" ht="78.5" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="G19" s="5" t="n"/>
+      <c r="H19" s="5" t="n"/>
+      <c r="I19" s="5" t="n"/>
+      <c r="J19" s="5" t="n"/>
+    </row>
+    <row r="20" ht="78.5" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>3. Set Up Your Server</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>3.11</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr"/>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="C20" s="5" t="n"/>
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>Look at your drives</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>1. Look at the picture of your server on the left. It shows every drive slot.
 2. Click one of the drives in the picture.
@@ -1382,68 +1417,68 @@
 4. Read the Issues box underneath it.</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>The number of drives in the picture matches the number you actually put in the server. Clicking a drive fills in Drive Properties with details about it. Issues says No issues found. in green.</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr"/>
-      <c r="H19" s="5" t="inlineStr"/>
-      <c r="I19" s="5" t="inlineStr"/>
-      <c r="J19" s="5" t="inlineStr"/>
-    </row>
-    <row r="20" ht="78.5" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="G20" s="5" t="n"/>
+      <c r="H20" s="5" t="n"/>
+      <c r="I20" s="5" t="n"/>
+      <c r="J20" s="5" t="n"/>
+    </row>
+    <row r="21" ht="78.5" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>3. Set Up Your Server</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>3.12</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr"/>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="C21" s="5" t="n"/>
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>Keep a spare copy of everything (only if you have 6 or more drives)</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>1. Find the tick box called Split Pools.
 2. If you have 6 or more drives, tick it and read the table that appears.
 3. If you have fewer than 6 drives, just check that the box is greyed out.</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>With 6 or more drives you can tick the box and a table appears showing a Storage row and a Backup row. With fewer than 6 drives the box is greyed out and the app explains why.</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr"/>
-      <c r="H20" s="5" t="inlineStr"/>
-      <c r="I20" s="5" t="inlineStr"/>
-      <c r="J20" s="5" t="inlineStr"/>
-    </row>
-    <row r="21" ht="107.5" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="G21" s="5" t="n"/>
+      <c r="H21" s="5" t="n"/>
+      <c r="I21" s="5" t="n"/>
+      <c r="J21" s="5" t="n"/>
+    </row>
+    <row r="22" ht="107.5" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>3. Set Up Your Server</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>3.13</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr"/>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>Check the Summary and start the setup</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>1. Click Next to reach the Summary page.
 2. Read everything on the page and check it matches what you typed.
@@ -1452,401 +1487,402 @@
 5. Click Complete Setup.</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>Everything on the Summary matches what you typed. Clicking Complete Setup starts a list of steps on a page called Setting Up Server.</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr"/>
-      <c r="H21" s="5" t="inlineStr"/>
-      <c r="I21" s="5" t="inlineStr"/>
-      <c r="J21" s="5" t="inlineStr"/>
-    </row>
-    <row r="22" ht="64" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="G22" s="5" t="n"/>
+      <c r="H22" s="5" t="n"/>
+      <c r="I22" s="5" t="n"/>
+      <c r="J22" s="5" t="n"/>
+    </row>
+    <row r="23" ht="64" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>3. Set Up Your Server</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>3.14</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr"/>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="C23" s="5" t="n"/>
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>Wait for all the green ticks</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>1. Watch the list of steps. Do not close the app.
 2. Wait until every step has finished.</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>Every step ends with a green tick. No step ends with a red cross. If you changed the Server Name, the server restarts itself afterwards and the app tells you this is normal.</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr"/>
-      <c r="H22" s="5" t="inlineStr"/>
-      <c r="I22" s="5" t="inlineStr"/>
-      <c r="J22" s="5" t="inlineStr"/>
-    </row>
-    <row r="23" ht="64" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="G23" s="5" t="n"/>
+      <c r="H23" s="5" t="n"/>
+      <c r="I23" s="5" t="n"/>
+      <c r="J23" s="5" t="n"/>
+    </row>
+    <row r="24" ht="93" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>3. Set Up Your Server</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>3.15</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr"/>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="C24" s="5" t="n"/>
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>The setup finishes</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>1. Read the message when everything is done.
-2. Find the two buttons at the bottom.</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>A message says you now have a network attached server you can start using immediately, and you see two buttons: Configure Backups and Setup More Storage Servers.</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="inlineStr"/>
-      <c r="H23" s="5" t="inlineStr"/>
-      <c r="I23" s="5" t="inlineStr"/>
-      <c r="J23" s="5" t="inlineStr"/>
-    </row>
-    <row r="24" ht="49.5" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
+2. Find the buttons at the bottom.
+3. Click Return to Dashboard.</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>A message says you now have a network attached server you can start using immediately, and you see three buttons: Return to Dashboard, Configure Backups and Setup More Storage Servers. Clicking Return to Dashboard takes you back to the Dashboard.</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="n"/>
+      <c r="H24" s="5" t="n"/>
+      <c r="I24" s="5" t="n"/>
+      <c r="J24" s="5" t="n"/>
+    </row>
+    <row r="25" ht="49.5" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>4. Check Your New Server</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>4.1</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr"/>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="C25" s="4" t="n"/>
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>Your server is on the Dashboard</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>1. Go back to the Dashboard.
 2. Find the box called Saved Servers.
 3. Find your server in the list.</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>Your server is listed with a green dot next to it, its name, and your user name and its address underneath.</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr"/>
-      <c r="H24" s="4" t="inlineStr"/>
-      <c r="I24" s="4" t="inlineStr"/>
-      <c r="J24" s="4" t="inlineStr"/>
-    </row>
-    <row r="25" ht="49.5" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="G25" s="4" t="n"/>
+      <c r="H25" s="4" t="n"/>
+      <c r="I25" s="4" t="n"/>
+      <c r="J25" s="4" t="n"/>
+    </row>
+    <row r="26" ht="49.5" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>4. Check Your New Server</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>4.2</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr"/>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="C26" s="5" t="n"/>
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>Click your server to see its details</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>1. Click once on your server's row.
 2. Look at the Storage and System Health boxes underneath.</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>The row is marked Viewing, and the Storage and System Health boxes fill in with information about your server.</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr"/>
-      <c r="H25" s="5" t="inlineStr"/>
-      <c r="I25" s="5" t="inlineStr"/>
-      <c r="J25" s="5" t="inlineStr"/>
-    </row>
-    <row r="26" ht="93" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="G26" s="5" t="n"/>
+      <c r="H26" s="5" t="n"/>
+      <c r="I26" s="5" t="n"/>
+      <c r="J26" s="5" t="n"/>
+    </row>
+    <row r="27" ht="93" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>4. Check Your New Server</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>4.3</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr"/>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="C27" s="5" t="n"/>
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>Open your new folder from your computer</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>1. Open your normal file browser (the one you use to look at your own files).
 2. Type in the folder address shown by Folder Preview earlier, for example \\myserver.local\data
 3. When asked, type the User Name and Password you wrote down.</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>The folder opens. It is empty to start with.</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr"/>
-      <c r="H26" s="5" t="inlineStr"/>
-      <c r="I26" s="5" t="inlineStr"/>
-      <c r="J26" s="5" t="inlineStr"/>
-    </row>
-    <row r="27" ht="35" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="G27" s="5" t="n"/>
+      <c r="H27" s="5" t="n"/>
+      <c r="I27" s="5" t="n"/>
+      <c r="J27" s="5" t="n"/>
+    </row>
+    <row r="28" ht="35" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>4. Check Your New Server</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr"/>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="C28" s="5" t="n"/>
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>Copy a file into your new folder</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>1. Drag any small file, such as a photo, into the folder.
 2. Open the file to check it still works.</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F28" s="5" t="inlineStr">
         <is>
           <t>The file copies over and opens normally.</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr"/>
-      <c r="H27" s="5" t="inlineStr"/>
-      <c r="I27" s="5" t="inlineStr"/>
-      <c r="J27" s="5" t="inlineStr"/>
-    </row>
-    <row r="28" ht="64" customHeight="1">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="G28" s="5" t="n"/>
+      <c r="H28" s="5" t="n"/>
+      <c r="I28" s="5" t="n"/>
+      <c r="J28" s="5" t="n"/>
+    </row>
+    <row r="29" ht="64" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>4. Check Your New Server</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr"/>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="C29" s="5" t="n"/>
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>The dot turns grey when the server is off</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>1. Turn the server off, or unplug its network cable.
 2. Go back to the Dashboard and wait a moment.
 3. Turn the server back on, or plug the cable back in, and wait again.</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="F29" s="5" t="inlineStr">
         <is>
           <t>The dot next to your server turns grey when it is off, and back to green when it is on again.</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr"/>
-      <c r="H28" s="5" t="inlineStr"/>
-      <c r="I28" s="5" t="inlineStr"/>
-      <c r="J28" s="5" t="inlineStr"/>
-    </row>
-    <row r="29" ht="49.5" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="G29" s="5" t="n"/>
+      <c r="H29" s="5" t="n"/>
+      <c r="I29" s="5" t="n"/>
+      <c r="J29" s="5" t="n"/>
+    </row>
+    <row r="30" ht="93" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>5. Set Up a Backup</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr"/>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="C30" s="4" t="n"/>
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>Open the Backup Manager</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>1. Go to the Dashboard.
 2. Click Manage Backups under Quick Actions.</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>The Backup Manager opens. Along the top you see two tabs: Local Backups and Remote Backups. Local Backups is already selected.</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr"/>
-      <c r="H29" s="4" t="inlineStr"/>
-      <c r="I29" s="4" t="inlineStr"/>
-      <c r="J29" s="4" t="inlineStr"/>
-    </row>
-    <row r="30" ht="35" customHeight="1">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>The Backup Manager opens. Along the top you see two tabs: Local Backups and Remote Backups. Local Backups is already selected. A short guided tour may appear the first time - read it or skip it; it does not come back afterwards.</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="n"/>
+      <c r="H30" s="4" t="n"/>
+      <c r="I30" s="4" t="n"/>
+      <c r="J30" s="4" t="n"/>
+    </row>
+    <row r="31" ht="35" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>5. Set Up a Backup</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>5.2</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr"/>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>Start a new backup</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>1. Make sure you are on the Local Backups tab.
 2. Click New Backup.</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>A page opens called Create Backup Task.</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr"/>
-      <c r="H30" s="5" t="inlineStr"/>
-      <c r="I30" s="5" t="inlineStr"/>
-      <c r="J30" s="5" t="inlineStr"/>
-    </row>
-    <row r="31" ht="78.5" customHeight="1">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="5" t="n"/>
+      <c r="I31" s="5" t="n"/>
+      <c r="J31" s="5" t="n"/>
+    </row>
+    <row r="32" ht="78.5" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>5. Set Up a Backup</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>5.3</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr"/>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="C32" s="5" t="n"/>
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>Choose where your files will be saved</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>1. Click the box called Back Up Location.
 2. Choose your server's folder. It looks like \\MyServer\data
 3. If it is not in the list, click the small refresh arrows next to the box and look again.</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="F32" s="5" t="inlineStr">
         <is>
           <t>Your folder appears in the list and you can choose it.</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr"/>
-      <c r="H31" s="5" t="inlineStr"/>
-      <c r="I31" s="5" t="inlineStr"/>
-      <c r="J31" s="5" t="inlineStr"/>
-    </row>
-    <row r="32" ht="35" customHeight="1">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="G32" s="5" t="n"/>
+      <c r="H32" s="5" t="n"/>
+      <c r="I32" s="5" t="n"/>
+      <c r="J32" s="5" t="n"/>
+    </row>
+    <row r="33" ht="35" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>5. Set Up a Backup</t>
         </is>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>5.4</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr"/>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="C33" s="5" t="n"/>
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>Choose how often to back up</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
         <is>
           <t>1. Leave Schedule Type set to Simple.
 2. Click Backup Interval and choose Hourly.</t>
         </is>
       </c>
-      <c r="F32" s="5" t="inlineStr">
+      <c r="F33" s="5" t="inlineStr">
         <is>
           <t>Hourly is now selected. Backups will run once every hour.</t>
         </is>
       </c>
-      <c r="G32" s="5" t="inlineStr"/>
-      <c r="H32" s="5" t="inlineStr"/>
-      <c r="I32" s="5" t="inlineStr"/>
-      <c r="J32" s="5" t="inlineStr"/>
-    </row>
-    <row r="33" ht="78.5" customHeight="1">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="G33" s="5" t="n"/>
+      <c r="H33" s="5" t="n"/>
+      <c r="I33" s="5" t="n"/>
+      <c r="J33" s="5" t="n"/>
+    </row>
+    <row r="34" ht="78.5" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>5. Set Up a Backup</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>5.5</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr"/>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="C34" s="5" t="n"/>
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>Choose which folders to back up</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>1. Find the + button under Folder Selection and click it.
 2. Pick a folder on your computer that has a few files in it.
@@ -1854,66 +1890,66 @@
 4. Give each one a short name you will recognise.</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="F34" s="5" t="inlineStr">
         <is>
           <t>Both folders appear in a list, each with its name and where it came from. The Next button is no longer greyed out.</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr"/>
-      <c r="H33" s="5" t="inlineStr"/>
-      <c r="I33" s="5" t="inlineStr"/>
-      <c r="J33" s="5" t="inlineStr"/>
-    </row>
-    <row r="34" ht="35" customHeight="1">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="G34" s="5" t="n"/>
+      <c r="H34" s="5" t="n"/>
+      <c r="I34" s="5" t="n"/>
+      <c r="J34" s="5" t="n"/>
+    </row>
+    <row r="35" ht="35" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>5. Set Up a Backup</t>
         </is>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>5.6</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr"/>
-      <c r="D34" s="5" t="inlineStr">
+      <c r="C35" s="5" t="n"/>
+      <c r="D35" s="5" t="inlineStr">
         <is>
           <t>The app stops you adding the same folder twice</t>
         </is>
       </c>
-      <c r="E34" s="5" t="inlineStr">
+      <c r="E35" s="5" t="inlineStr">
         <is>
           <t>1. Click + and try to add a folder that is already in the list.</t>
         </is>
       </c>
-      <c r="F34" s="5" t="inlineStr">
+      <c r="F35" s="5" t="inlineStr">
         <is>
           <t>A message appears saying This path is already added. The folder is not added twice.</t>
         </is>
       </c>
-      <c r="G34" s="5" t="inlineStr"/>
-      <c r="H34" s="5" t="inlineStr"/>
-      <c r="I34" s="5" t="inlineStr"/>
-      <c r="J34" s="5" t="inlineStr"/>
-    </row>
-    <row r="35" ht="78.5" customHeight="1">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="G35" s="5" t="n"/>
+      <c r="H35" s="5" t="n"/>
+      <c r="I35" s="5" t="n"/>
+      <c r="J35" s="5" t="n"/>
+    </row>
+    <row r="36" ht="78.5" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>5. Set Up a Backup</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>5.7</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr"/>
-      <c r="D35" s="5" t="inlineStr">
+      <c r="C36" s="5" t="n"/>
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>Sign in to your folder</t>
         </is>
       </c>
-      <c r="E35" s="5" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>1. Click Next to reach the Samba Login page.
 2. Type the WRONG password on purpose and click Next.
@@ -1921,68 +1957,68 @@
 4. Click Next.</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
+      <c r="F36" s="5" t="inlineStr">
         <is>
           <t>The wrong password gives a red message saying Invalid credentials. Please check your username and password. The correct one lets you carry on to the Summary page.</t>
         </is>
       </c>
-      <c r="G35" s="5" t="inlineStr"/>
-      <c r="H35" s="5" t="inlineStr"/>
-      <c r="I35" s="5" t="inlineStr"/>
-      <c r="J35" s="5" t="inlineStr"/>
-    </row>
-    <row r="36" ht="78.5" customHeight="1">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="G36" s="5" t="n"/>
+      <c r="H36" s="5" t="n"/>
+      <c r="I36" s="5" t="n"/>
+      <c r="J36" s="5" t="n"/>
+    </row>
+    <row r="37" ht="93" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>5. Set Up a Backup</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>5.8</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr"/>
-      <c r="D36" s="5" t="inlineStr">
+      <c r="C37" s="5" t="n"/>
+      <c r="D37" s="5" t="inlineStr">
         <is>
           <t>Type your computer password when asked (Linux only)</t>
         </is>
       </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>1. On the Summary screen, read the yellow message about your admin password.
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>1. On the Summary screen, read the coloured message at the top.
 2. Finish the wizard.
-3. When a box asks for your computer's password, type it and click OK.</t>
-        </is>
-      </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>The message explains why the password is needed, the box appears, and the backup is created after you type it.</t>
-        </is>
-      </c>
-      <c r="G36" s="5" t="inlineStr"/>
-      <c r="H36" s="5" t="inlineStr"/>
-      <c r="I36" s="5" t="inlineStr"/>
-      <c r="J36" s="5" t="inlineStr"/>
-    </row>
-    <row r="37" ht="78.5" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
+3. When a box asks for your computer's admin password, type it and click OK.</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>The message says: Note: On Linux, if this is your first backup, you will be prompted for your admin password to set up the server connection. The box appears, and after you type the password the backup is created. You are only asked once.</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="n"/>
+      <c r="H37" s="5" t="n"/>
+      <c r="I37" s="5" t="n"/>
+      <c r="J37" s="5" t="n"/>
+    </row>
+    <row r="38" ht="78.5" customHeight="1">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>5. Set Up a Backup</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>5.9</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr"/>
-      <c r="D37" s="5" t="inlineStr">
+      <c r="C38" s="5" t="n"/>
+      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>Check the Summary and finish</t>
         </is>
       </c>
-      <c r="E37" s="5" t="inlineStr">
+      <c r="E38" s="5" t="inlineStr">
         <is>
           <t>1. Read the Summary page. Check the folders and the timing are what you chose.
 2. Click Next.
@@ -1990,199 +2026,233 @@
 4. Click Go To Backup Manager.</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
+      <c r="F38" s="5" t="inlineStr">
         <is>
           <t>The last page says Complete! Your Backup Plan is Now Active. Clicking the button takes you back to the list of backups.</t>
         </is>
       </c>
-      <c r="G37" s="5" t="inlineStr"/>
-      <c r="H37" s="5" t="inlineStr"/>
-      <c r="I37" s="5" t="inlineStr"/>
-      <c r="J37" s="5" t="inlineStr"/>
-    </row>
-    <row r="38" ht="49.5" customHeight="1">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="G38" s="5" t="n"/>
+      <c r="H38" s="5" t="n"/>
+      <c r="I38" s="5" t="n"/>
+      <c r="J38" s="5" t="n"/>
+    </row>
+    <row r="39" ht="107.5" customHeight="1">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>5. Set Up a Backup</t>
         </is>
       </c>
-      <c r="B38" s="5" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>5.10</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr"/>
-      <c r="D38" s="5" t="inlineStr">
+      <c r="C39" s="5" t="n"/>
+      <c r="D39" s="5" t="inlineStr">
         <is>
           <t>Your backup is in the list</t>
         </is>
       </c>
-      <c r="E38" s="5" t="inlineStr">
+      <c r="E39" s="5" t="inlineStr">
         <is>
           <t>1. Look at the table on the Local Backups tab.
 2. Find your new backups.</t>
         </is>
       </c>
-      <c r="F38" s="5" t="inlineStr">
-        <is>
-          <t>Your backups are listed with the name you gave them, the folder they came from, where they are going, how often they run, and when they will run next.</t>
-        </is>
-      </c>
-      <c r="G38" s="5" t="inlineStr"/>
-      <c r="H38" s="5" t="inlineStr"/>
-      <c r="I38" s="5" t="inlineStr"/>
-      <c r="J38" s="5" t="inlineStr"/>
-    </row>
-    <row r="39" ht="49.5" customHeight="1">
-      <c r="A39" s="4" t="inlineStr">
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>Your backups are listed with the name you gave them, the user name, the folder they came from, where they are going, how often they run, a Status badge with a coloured dot, when they last ran, when they will run next, and an Enabled switch. Underneath the table a line counts them up, for example 2 backups · 2 online.</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="n"/>
+      <c r="H39" s="5" t="n"/>
+      <c r="I39" s="5" t="n"/>
+      <c r="J39" s="5" t="n"/>
+    </row>
+    <row r="40" ht="78.5" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>6. Run a Backup and Check It</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>6.1</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr"/>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="C40" s="4" t="n"/>
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t>Back up now instead of waiting</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="E40" s="4" t="inlineStr">
         <is>
           <t>1. Click on one of your backups to select it.
 2. Click Run Now.</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>The backup starts straight away. A panel appears at the bottom of the screen showing how far along it is.</t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="inlineStr"/>
-      <c r="H39" s="4" t="inlineStr"/>
-      <c r="I39" s="4" t="inlineStr"/>
-      <c r="J39" s="4" t="inlineStr"/>
-    </row>
-    <row r="40" ht="35" customHeight="1">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>The backup starts straight away. A panel appears at the bottom of the screen saying 1 backup in progress, with a bar showing how far along it is and the name of the task.</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="n"/>
+      <c r="H40" s="4" t="n"/>
+      <c r="I40" s="4" t="n"/>
+      <c r="J40" s="4" t="n"/>
+    </row>
+    <row r="41" ht="35" customHeight="1">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>6. Run a Backup and Check It</t>
         </is>
       </c>
-      <c r="B40" s="5" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>6.2</t>
         </is>
       </c>
-      <c r="C40" s="5" t="inlineStr"/>
-      <c r="D40" s="5" t="inlineStr">
+      <c r="C41" s="5" t="n"/>
+      <c r="D41" s="5" t="inlineStr">
         <is>
           <t>Wait for it to finish</t>
         </is>
       </c>
-      <c r="E40" s="5" t="inlineStr">
+      <c r="E41" s="5" t="inlineStr">
         <is>
           <t>1. Watch the bar at the bottom until it finishes.</t>
         </is>
       </c>
-      <c r="F40" s="5" t="inlineStr">
+      <c r="F41" s="5" t="inlineStr">
         <is>
           <t>The bar fills up and the backup finishes. The app says it worked. Nothing crashes.</t>
         </is>
       </c>
-      <c r="G40" s="5" t="inlineStr"/>
-      <c r="H40" s="5" t="inlineStr"/>
-      <c r="I40" s="5" t="inlineStr"/>
-      <c r="J40" s="5" t="inlineStr"/>
-    </row>
-    <row r="41" ht="49.5" customHeight="1">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="G41" s="5" t="n"/>
+      <c r="H41" s="5" t="n"/>
+      <c r="I41" s="5" t="n"/>
+      <c r="J41" s="5" t="n"/>
+    </row>
+    <row r="42" ht="93" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>6. Run a Backup and Check It</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>6.3</t>
         </is>
       </c>
-      <c r="C41" s="5" t="inlineStr"/>
-      <c r="D41" s="5" t="inlineStr">
+      <c r="C42" s="5" t="n"/>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Watch the Status badge</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>1. While a backup is running, look at the Status column on its row.
+2. Wait for it to finish and look again.
+3. Look at the line underneath the table.</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>While it runs the badge says Running with a blue dot. When it finishes the badge goes back to Online with a green dot. If something went wrong it says Failed in red. The line under the table counts your backups, for example 2 backups · 2 online.</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="n"/>
+      <c r="H42" s="5" t="n"/>
+      <c r="I42" s="5" t="n"/>
+      <c r="J42" s="5" t="n"/>
+    </row>
+    <row r="43" ht="49.5" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>6. Run a Backup and Check It</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>6.4</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="n"/>
+      <c r="D43" s="5" t="inlineStr">
         <is>
           <t>Your files really are on the server</t>
         </is>
       </c>
-      <c r="E41" s="5" t="inlineStr">
+      <c r="E43" s="5" t="inlineStr">
         <is>
           <t>1. Open your network folder from your computer again.
 2. Look for the folders you backed up.
 3. Open one or two of the files.</t>
         </is>
       </c>
-      <c r="F41" s="5" t="inlineStr">
+      <c r="F43" s="5" t="inlineStr">
         <is>
           <t>All of your files are there and they open normally.</t>
         </is>
       </c>
-      <c r="G41" s="5" t="inlineStr"/>
-      <c r="H41" s="5" t="inlineStr"/>
-      <c r="I41" s="5" t="inlineStr"/>
-      <c r="J41" s="5" t="inlineStr"/>
-    </row>
-    <row r="42" ht="35" customHeight="1">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="G43" s="5" t="n"/>
+      <c r="H43" s="5" t="n"/>
+      <c r="I43" s="5" t="n"/>
+      <c r="J43" s="5" t="n"/>
+    </row>
+    <row r="44" ht="35" customHeight="1">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>6. Run a Backup and Check It</t>
         </is>
       </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>6.4</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr"/>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="n"/>
+      <c r="D44" s="5" t="inlineStr">
         <is>
           <t>Look at the backup history</t>
         </is>
       </c>
-      <c r="E42" s="5" t="inlineStr">
+      <c r="E44" s="5" t="inlineStr">
         <is>
           <t>1. Select the backup in the list.
 2. Click Logs.</t>
         </is>
       </c>
-      <c r="F42" s="5" t="inlineStr">
+      <c r="F44" s="5" t="inlineStr">
         <is>
           <t>A list appears showing each time the backup ran, with the date and time, and whether it worked.</t>
         </is>
       </c>
-      <c r="G42" s="5" t="inlineStr"/>
-      <c r="H42" s="5" t="inlineStr"/>
-      <c r="I42" s="5" t="inlineStr"/>
-      <c r="J42" s="5" t="inlineStr"/>
-    </row>
-    <row r="43" ht="64" customHeight="1">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="G44" s="5" t="n"/>
+      <c r="H44" s="5" t="n"/>
+      <c r="I44" s="5" t="n"/>
+      <c r="J44" s="5" t="n"/>
+    </row>
+    <row r="45" ht="64" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>6. Run a Backup and Check It</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>6.5</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr"/>
-      <c r="D43" s="5" t="inlineStr">
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>6.6</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="n"/>
+      <c r="D45" s="5" t="inlineStr">
         <is>
           <t>A backup runs on its own</t>
         </is>
       </c>
-      <c r="E43" s="5" t="inlineStr">
+      <c r="E45" s="5" t="inlineStr">
         <is>
           <t>1. Add a new file to one of the folders you are backing up.
 2. Leave the app alone until the next hour has passed.
@@ -2190,102 +2260,177 @@
 4. Look in your network folder for the new file.</t>
         </is>
       </c>
-      <c r="F43" s="5" t="inlineStr">
+      <c r="F45" s="5" t="inlineStr">
         <is>
           <t>The backup ran by itself without you doing anything, and the new file is on the server.</t>
         </is>
       </c>
-      <c r="G43" s="5" t="inlineStr"/>
-      <c r="H43" s="5" t="inlineStr"/>
-      <c r="I43" s="5" t="inlineStr"/>
-      <c r="J43" s="5" t="inlineStr"/>
-    </row>
-    <row r="44" ht="64" customHeight="1">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="G45" s="5" t="n"/>
+      <c r="H45" s="5" t="n"/>
+      <c r="I45" s="5" t="n"/>
+      <c r="J45" s="5" t="n"/>
+    </row>
+    <row r="46" ht="107.5" customHeight="1">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>6. Run a Backup and Check It</t>
         </is>
       </c>
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t>6.6</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr"/>
-      <c r="D44" s="5" t="inlineStr">
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>6.7</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="n"/>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Backups still run when the app is closed</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>1. Make sure one of your backups is set to Hourly.
+2. Put a new file in the folder that is being backed up.
+3. Close the 45Drives Storage Wizard completely.
+4. Wait until the next hour has passed.
+5. Open the app again and look at the Last Run column.
+6. Look in your network folder for the new file.</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>Last Run shows that the backup ran while the app was closed, and the new file is on the server.</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="n"/>
+      <c r="H46" s="5" t="n"/>
+      <c r="I46" s="5" t="n"/>
+      <c r="J46" s="5" t="n"/>
+    </row>
+    <row r="47" ht="136.5" customHeight="1">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>6. Run a Backup and Check It</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>6.8</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="n"/>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Backups still run when you are signed out</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>1. Make sure one of your backups is set to Hourly.
+2. Put a new file in the folder that is being backed up.
+3. Sign out of your computer. Do not shut it down.
+4. Wait until the next hour has passed.
+5. Sign back in and open the app.
+6. Look at the Last Run column, then select the backup and click Logs.
+7. Look in your network folder for the new file.</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>Last Run shows that the backup ran while you were signed out, the Logs show it finished successfully, and the new file is on the server.</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="n"/>
+      <c r="H47" s="5" t="n"/>
+      <c r="I47" s="5" t="n"/>
+      <c r="J47" s="5" t="n"/>
+    </row>
+    <row r="48" ht="64" customHeight="1">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>6. Run a Backup and Check It</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>6.9</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="n"/>
+      <c r="D48" s="5" t="inlineStr">
         <is>
           <t>It tells you clearly if the server is off</t>
         </is>
       </c>
-      <c r="E44" s="5" t="inlineStr">
+      <c r="E48" s="5" t="inlineStr">
         <is>
           <t>1. Turn the server off.
 2. Select the backup and click Run Now.
 3. Turn the server back on and click Run Now again.</t>
         </is>
       </c>
-      <c r="F44" s="5" t="inlineStr">
+      <c r="F48" s="5" t="inlineStr">
         <is>
           <t>The app tells you in plain words that it could not reach the server. The app does not freeze or close. Once the server is back on, the backup works again.</t>
         </is>
       </c>
-      <c r="G44" s="5" t="inlineStr"/>
-      <c r="H44" s="5" t="inlineStr"/>
-      <c r="I44" s="5" t="inlineStr"/>
-      <c r="J44" s="5" t="inlineStr"/>
-    </row>
-    <row r="45" ht="49.5" customHeight="1">
-      <c r="A45" s="4" t="inlineStr">
+      <c r="G48" s="5" t="n"/>
+      <c r="H48" s="5" t="n"/>
+      <c r="I48" s="5" t="n"/>
+      <c r="J48" s="5" t="n"/>
+    </row>
+    <row r="49" ht="49.5" customHeight="1">
+      <c r="A49" s="4" t="inlineStr">
         <is>
           <t>7. Get a File Back</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>7.1</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr"/>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="C49" s="4" t="n"/>
+      <c r="D49" s="4" t="inlineStr">
         <is>
           <t>Delete a file on purpose</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="E49" s="4" t="inlineStr">
         <is>
           <t>1. Pick one file inside a folder you have backed up.
 2. Note its name.
 3. Delete it from your computer.</t>
         </is>
       </c>
-      <c r="F45" s="4" t="inlineStr">
+      <c r="F49" s="4" t="inlineStr">
         <is>
           <t>The file is gone from your computer.</t>
         </is>
       </c>
-      <c r="G45" s="4" t="inlineStr"/>
-      <c r="H45" s="4" t="inlineStr"/>
-      <c r="I45" s="4" t="inlineStr"/>
-      <c r="J45" s="4" t="inlineStr"/>
-    </row>
-    <row r="46" ht="64" customHeight="1">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="G49" s="4" t="n"/>
+      <c r="H49" s="4" t="n"/>
+      <c r="I49" s="4" t="n"/>
+      <c r="J49" s="4" t="n"/>
+    </row>
+    <row r="50" ht="64" customHeight="1">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>7. Get a File Back</t>
         </is>
       </c>
-      <c r="B46" s="5" t="inlineStr">
+      <c r="B50" s="5" t="inlineStr">
         <is>
           <t>7.2</t>
         </is>
       </c>
-      <c r="C46" s="5" t="inlineStr"/>
-      <c r="D46" s="5" t="inlineStr">
+      <c r="C50" s="5" t="n"/>
+      <c r="D50" s="5" t="inlineStr">
         <is>
           <t>Find the file in your backup</t>
         </is>
       </c>
-      <c r="E46" s="5" t="inlineStr">
+      <c r="E50" s="5" t="inlineStr">
         <is>
           <t>1. Go to the Backup Manager, Local Backups tab.
 2. Select the backup that had the file in it.
@@ -2293,34 +2438,34 @@
 4. Click through the folders until you find the file.</t>
         </is>
       </c>
-      <c r="F46" s="5" t="inlineStr">
+      <c r="F50" s="5" t="inlineStr">
         <is>
           <t>You can see the folders and files that were backed up, and you can click into folders and back out again.</t>
         </is>
       </c>
-      <c r="G46" s="5" t="inlineStr"/>
-      <c r="H46" s="5" t="inlineStr"/>
-      <c r="I46" s="5" t="inlineStr"/>
-      <c r="J46" s="5" t="inlineStr"/>
-    </row>
-    <row r="47" ht="64" customHeight="1">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="G50" s="5" t="n"/>
+      <c r="H50" s="5" t="n"/>
+      <c r="I50" s="5" t="n"/>
+      <c r="J50" s="5" t="n"/>
+    </row>
+    <row r="51" ht="64" customHeight="1">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>7. Get a File Back</t>
         </is>
       </c>
-      <c r="B47" s="5" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>7.3</t>
         </is>
       </c>
-      <c r="C47" s="5" t="inlineStr"/>
-      <c r="D47" s="5" t="inlineStr">
+      <c r="C51" s="5" t="n"/>
+      <c r="D51" s="5" t="inlineStr">
         <is>
           <t>Bring the file back</t>
         </is>
       </c>
-      <c r="E47" s="5" t="inlineStr">
+      <c r="E51" s="5" t="inlineStr">
         <is>
           <t>1. Select the file.
 2. Restore it.
@@ -2328,68 +2473,68 @@
 4. Open it.</t>
         </is>
       </c>
-      <c r="F47" s="5" t="inlineStr">
+      <c r="F51" s="5" t="inlineStr">
         <is>
           <t>The file comes back to your computer and opens exactly as it did before.</t>
         </is>
       </c>
-      <c r="G47" s="5" t="inlineStr"/>
-      <c r="H47" s="5" t="inlineStr"/>
-      <c r="I47" s="5" t="inlineStr"/>
-      <c r="J47" s="5" t="inlineStr"/>
-    </row>
-    <row r="48" ht="64" customHeight="1">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="G51" s="5" t="n"/>
+      <c r="H51" s="5" t="n"/>
+      <c r="I51" s="5" t="n"/>
+      <c r="J51" s="5" t="n"/>
+    </row>
+    <row r="52" ht="64" customHeight="1">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>7. Get a File Back</t>
         </is>
       </c>
-      <c r="B48" s="5" t="inlineStr">
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>7.4</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr"/>
-      <c r="D48" s="5" t="inlineStr">
+      <c r="C52" s="5" t="n"/>
+      <c r="D52" s="5" t="inlineStr">
         <is>
           <t>Bring a whole folder back</t>
         </is>
       </c>
-      <c r="E48" s="5" t="inlineStr">
+      <c r="E52" s="5" t="inlineStr">
         <is>
           <t>1. In View/Restore, choose a whole folder instead of one file.
 2. Restore it.
 3. Look at what came back.</t>
         </is>
       </c>
-      <c r="F48" s="5" t="inlineStr">
+      <c r="F52" s="5" t="inlineStr">
         <is>
           <t>Everything inside the folder comes back, in the right folders, and the files open normally.</t>
         </is>
       </c>
-      <c r="G48" s="5" t="inlineStr"/>
-      <c r="H48" s="5" t="inlineStr"/>
-      <c r="I48" s="5" t="inlineStr"/>
-      <c r="J48" s="5" t="inlineStr"/>
-    </row>
-    <row r="49" ht="78.5" customHeight="1">
-      <c r="A49" s="4" t="inlineStr">
+      <c r="G52" s="5" t="n"/>
+      <c r="H52" s="5" t="n"/>
+      <c r="I52" s="5" t="n"/>
+      <c r="J52" s="5" t="n"/>
+    </row>
+    <row r="53" ht="78.5" customHeight="1">
+      <c r="A53" s="4" t="inlineStr">
         <is>
           <t>8. Make the App Yours</t>
         </is>
       </c>
-      <c r="B49" s="4" t="inlineStr">
+      <c r="B53" s="4" t="inlineStr">
         <is>
           <t>8.1</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr"/>
-      <c r="D49" s="4" t="inlineStr">
+      <c r="C53" s="4" t="n"/>
+      <c r="D53" s="4" t="inlineStr">
         <is>
           <t>Change the colour</t>
         </is>
       </c>
-      <c r="E49" s="4" t="inlineStr">
+      <c r="E53" s="4" t="inlineStr">
         <is>
           <t>1. Open the menu (the three lines in the top-right corner).
 2. Under Appearance, click 45Drives.
@@ -2398,34 +2543,34 @@
 5. Then click 45Studio.</t>
         </is>
       </c>
-      <c r="F49" s="4" t="inlineStr">
+      <c r="F53" s="4" t="inlineStr">
         <is>
           <t>The whole app changes colour each time. Words stay easy to read on every colour.</t>
         </is>
       </c>
-      <c r="G49" s="4" t="inlineStr"/>
-      <c r="H49" s="4" t="inlineStr"/>
-      <c r="I49" s="4" t="inlineStr"/>
-      <c r="J49" s="4" t="inlineStr"/>
-    </row>
-    <row r="50" ht="78.5" customHeight="1">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="G53" s="4" t="n"/>
+      <c r="H53" s="4" t="n"/>
+      <c r="I53" s="4" t="n"/>
+      <c r="J53" s="4" t="n"/>
+    </row>
+    <row r="54" ht="78.5" customHeight="1">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>8. Make the App Yours</t>
         </is>
       </c>
-      <c r="B50" s="5" t="inlineStr">
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>8.2</t>
         </is>
       </c>
-      <c r="C50" s="5" t="inlineStr"/>
-      <c r="D50" s="5" t="inlineStr">
+      <c r="C54" s="5" t="n"/>
+      <c r="D54" s="5" t="inlineStr">
         <is>
           <t>Try dark mode</t>
         </is>
       </c>
-      <c r="E50" s="5" t="inlineStr">
+      <c r="E54" s="5" t="inlineStr">
         <is>
           <t>1. In the menu, find the Light / Dark switch next to the colours.
 2. Switch it to Dark.
@@ -2433,68 +2578,68 @@
 4. Switch it back to Light.</t>
         </is>
       </c>
-      <c r="F50" s="5" t="inlineStr">
+      <c r="F54" s="5" t="inlineStr">
         <is>
           <t>The app goes dark and then light again. Words stay easy to read both ways.</t>
         </is>
       </c>
-      <c r="G50" s="5" t="inlineStr"/>
-      <c r="H50" s="5" t="inlineStr"/>
-      <c r="I50" s="5" t="inlineStr"/>
-      <c r="J50" s="5" t="inlineStr"/>
-    </row>
-    <row r="51" ht="49.5" customHeight="1">
-      <c r="A51" s="5" t="inlineStr">
+      <c r="G54" s="5" t="n"/>
+      <c r="H54" s="5" t="n"/>
+      <c r="I54" s="5" t="n"/>
+      <c r="J54" s="5" t="n"/>
+    </row>
+    <row r="55" ht="49.5" customHeight="1">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>8. Make the App Yours</t>
         </is>
       </c>
-      <c r="B51" s="5" t="inlineStr">
+      <c r="B55" s="5" t="inlineStr">
         <is>
           <t>8.3</t>
         </is>
       </c>
-      <c r="C51" s="5" t="inlineStr"/>
-      <c r="D51" s="5" t="inlineStr">
+      <c r="C55" s="5" t="n"/>
+      <c r="D55" s="5" t="inlineStr">
         <is>
           <t>The app remembers your choice</t>
         </is>
       </c>
-      <c r="E51" s="5" t="inlineStr">
+      <c r="E55" s="5" t="inlineStr">
         <is>
           <t>1. Pick a colour and Dark mode.
 2. Close the app completely.
 3. Open it again.</t>
         </is>
       </c>
-      <c r="F51" s="5" t="inlineStr">
+      <c r="F55" s="5" t="inlineStr">
         <is>
           <t>The app opens with the colour and the light/dark setting you chose.</t>
         </is>
       </c>
-      <c r="G51" s="5" t="inlineStr"/>
-      <c r="H51" s="5" t="inlineStr"/>
-      <c r="I51" s="5" t="inlineStr"/>
-      <c r="J51" s="5" t="inlineStr"/>
-    </row>
-    <row r="52" ht="107.5" customHeight="1">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="G55" s="5" t="n"/>
+      <c r="H55" s="5" t="n"/>
+      <c r="I55" s="5" t="n"/>
+      <c r="J55" s="5" t="n"/>
+    </row>
+    <row r="56" ht="107.5" customHeight="1">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>8. Make the App Yours</t>
         </is>
       </c>
-      <c r="B52" s="5" t="inlineStr">
+      <c r="B56" s="5" t="inlineStr">
         <is>
           <t>8.4</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr"/>
-      <c r="D52" s="5" t="inlineStr">
+      <c r="C56" s="5" t="n"/>
+      <c r="D56" s="5" t="inlineStr">
         <is>
           <t>Give your server a friendly name</t>
         </is>
       </c>
-      <c r="E52" s="5" t="inlineStr">
+      <c r="E56" s="5" t="inlineStr">
         <is>
           <t>1. Open the menu and click Settings.
 2. On the left, click Servers, then Saved.
@@ -2505,102 +2650,137 @@
 7. Go back to the Dashboard.</t>
         </is>
       </c>
-      <c r="F52" s="5" t="inlineStr">
+      <c r="F56" s="5" t="inlineStr">
         <is>
           <t>Your friendly name is shown on the Dashboard instead of the old one, and a gold star appears next to it.</t>
         </is>
       </c>
-      <c r="G52" s="5" t="inlineStr"/>
-      <c r="H52" s="5" t="inlineStr"/>
-      <c r="I52" s="5" t="inlineStr"/>
-      <c r="J52" s="5" t="inlineStr"/>
-    </row>
-    <row r="53" ht="49.5" customHeight="1">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="G56" s="5" t="n"/>
+      <c r="H56" s="5" t="n"/>
+      <c r="I56" s="5" t="n"/>
+      <c r="J56" s="5" t="n"/>
+    </row>
+    <row r="57" ht="49.5" customHeight="1">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>8. Make the App Yours</t>
         </is>
       </c>
-      <c r="B53" s="5" t="inlineStr">
+      <c r="B57" s="5" t="inlineStr">
         <is>
           <t>8.5</t>
         </is>
       </c>
-      <c r="C53" s="5" t="inlineStr"/>
-      <c r="D53" s="5" t="inlineStr">
+      <c r="C57" s="5" t="n"/>
+      <c r="D57" s="5" t="inlineStr">
         <is>
           <t>Your settings survive closing the app</t>
         </is>
       </c>
-      <c r="E53" s="5" t="inlineStr">
+      <c r="E57" s="5" t="inlineStr">
         <is>
           <t>1. Close the app completely.
 2. Open it again.
 3. Look at the Dashboard.</t>
         </is>
       </c>
-      <c r="F53" s="5" t="inlineStr">
+      <c r="F57" s="5" t="inlineStr">
         <is>
           <t>Your friendly name, the gold star, your colour and your backups are all still there.</t>
         </is>
       </c>
-      <c r="G53" s="5" t="inlineStr"/>
-      <c r="H53" s="5" t="inlineStr"/>
-      <c r="I53" s="5" t="inlineStr"/>
-      <c r="J53" s="5" t="inlineStr"/>
-    </row>
-    <row r="54" ht="49.5" customHeight="1">
-      <c r="A54" s="4" t="inlineStr">
+      <c r="G57" s="5" t="n"/>
+      <c r="H57" s="5" t="n"/>
+      <c r="I57" s="5" t="n"/>
+      <c r="J57" s="5" t="n"/>
+    </row>
+    <row r="58" ht="78.5" customHeight="1">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>8. Make the App Yours</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>8.6</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="n"/>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Turn the guided tours back on</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>1. Open the menu and click Settings.
+2. On the left, under Client, click Display.
+3. Find Reset guided tours and click Reset.
+4. Close Settings and go to the Dashboard.</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>A message says Guided tours have been reset. The walkthrough appears again the next time you open the Dashboard and the Backup Manager.</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="n"/>
+      <c r="H58" s="5" t="n"/>
+      <c r="I58" s="5" t="n"/>
+      <c r="J58" s="5" t="n"/>
+    </row>
+    <row r="59" ht="49.5" customHeight="1">
+      <c r="A59" s="4" t="inlineStr">
         <is>
           <t>9. Tidy Up</t>
         </is>
       </c>
-      <c r="B54" s="4" t="inlineStr">
+      <c r="B59" s="4" t="inlineStr">
         <is>
           <t>9.1</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr"/>
-      <c r="D54" s="4" t="inlineStr">
+      <c r="C59" s="4" t="n"/>
+      <c r="D59" s="4" t="inlineStr">
         <is>
           <t>See what has been happening</t>
         </is>
       </c>
-      <c r="E54" s="4" t="inlineStr">
+      <c r="E59" s="4" t="inlineStr">
         <is>
           <t>1. Go to the Dashboard.
 2. Look at the box called Recent Activity.
 3. Look at Upcoming Backups on the right-hand side.</t>
         </is>
       </c>
-      <c r="F54" s="4" t="inlineStr">
+      <c r="F59" s="4" t="inlineStr">
         <is>
           <t>Recent Activity lists the backups that have run, with a green dot for ones that worked. Upcoming Backups shows when the next one will run.</t>
         </is>
       </c>
-      <c r="G54" s="4" t="inlineStr"/>
-      <c r="H54" s="4" t="inlineStr"/>
-      <c r="I54" s="4" t="inlineStr"/>
-      <c r="J54" s="4" t="inlineStr"/>
-    </row>
-    <row r="55" ht="93" customHeight="1">
-      <c r="A55" s="5" t="inlineStr">
+      <c r="G59" s="4" t="n"/>
+      <c r="H59" s="4" t="n"/>
+      <c r="I59" s="4" t="n"/>
+      <c r="J59" s="4" t="n"/>
+    </row>
+    <row r="60" ht="93" customHeight="1">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>9. Tidy Up</t>
         </is>
       </c>
-      <c r="B55" s="5" t="inlineStr">
+      <c r="B60" s="5" t="inlineStr">
         <is>
           <t>9.2</t>
         </is>
       </c>
-      <c r="C55" s="5" t="inlineStr"/>
-      <c r="D55" s="5" t="inlineStr">
+      <c r="C60" s="5" t="n"/>
+      <c r="D60" s="5" t="inlineStr">
         <is>
           <t>Turn a backup off and on</t>
         </is>
       </c>
-      <c r="E55" s="5" t="inlineStr">
+      <c r="E60" s="5" t="inlineStr">
         <is>
           <t>1. In the Backup Manager, find the Enabled switch on the end of your backup's row.
 2. Switch it off.
@@ -2608,84 +2788,156 @@
 4. Switch it back on.</t>
         </is>
       </c>
-      <c r="F55" s="5" t="inlineStr">
+      <c r="F60" s="5" t="inlineStr">
         <is>
           <t>While the switch is off, the backup does not run. Switching it back on makes it run again on schedule.</t>
         </is>
       </c>
-      <c r="G55" s="5" t="inlineStr"/>
-      <c r="H55" s="5" t="inlineStr"/>
-      <c r="I55" s="5" t="inlineStr"/>
-      <c r="J55" s="5" t="inlineStr"/>
-    </row>
-    <row r="56" ht="49.5" customHeight="1">
-      <c r="A56" s="5" t="inlineStr">
+      <c r="G60" s="5" t="n"/>
+      <c r="H60" s="5" t="n"/>
+      <c r="I60" s="5" t="n"/>
+      <c r="J60" s="5" t="n"/>
+    </row>
+    <row r="61" ht="107.5" customHeight="1">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>9. Tidy Up</t>
         </is>
       </c>
-      <c r="B56" s="5" t="inlineStr">
+      <c r="B61" s="5" t="inlineStr">
         <is>
           <t>9.3</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr"/>
-      <c r="D56" s="5" t="inlineStr">
+      <c r="C61" s="5" t="n"/>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Change a backup you already made</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>1. In the Backup Manager, click one backup to select it.
+2. Click Edit.
+3. Change the Backup Name to something else.
+4. Leave Samba Username and Samba Password empty.
+5. Click Save Changes.
+6. Select the backup again and click Run Now.</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>The box says Leave both blank to keep the saved ones. The change is saved without asking you to type a password again, the new name appears in the list, and the backup still runs successfully.</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="n"/>
+      <c r="H61" s="5" t="n"/>
+      <c r="I61" s="5" t="n"/>
+      <c r="J61" s="5" t="n"/>
+    </row>
+    <row r="62" ht="49.5" customHeight="1">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>9. Tidy Up</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="n"/>
+      <c r="D62" s="5" t="inlineStr">
         <is>
           <t>Delete a backup you do not want</t>
         </is>
       </c>
-      <c r="E56" s="5" t="inlineStr">
+      <c r="E62" s="5" t="inlineStr">
         <is>
           <t>1. Select a backup.
 2. Click the bin icon.
 3. Confirm.</t>
         </is>
       </c>
-      <c r="F56" s="5" t="inlineStr">
+      <c r="F62" s="5" t="inlineStr">
         <is>
           <t>The backup disappears from the list and does not run again.</t>
         </is>
       </c>
-      <c r="G56" s="5" t="inlineStr"/>
-      <c r="H56" s="5" t="inlineStr"/>
-      <c r="I56" s="5" t="inlineStr"/>
-      <c r="J56" s="5" t="inlineStr"/>
-    </row>
-    <row r="57" ht="35" customHeight="1">
-      <c r="A57" s="5" t="inlineStr">
+      <c r="G62" s="5" t="n"/>
+      <c r="H62" s="5" t="n"/>
+      <c r="I62" s="5" t="n"/>
+      <c r="J62" s="5" t="n"/>
+    </row>
+    <row r="63" ht="93" customHeight="1">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>9. Tidy Up</t>
         </is>
       </c>
-      <c r="B57" s="5" t="inlineStr">
-        <is>
-          <t>9.4</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr"/>
-      <c r="D57" s="5" t="inlineStr">
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="n"/>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Remove a server you no longer use</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>1. Open the menu and click Settings.
+2. On the left, under Servers, click Saved.
+3. Find a server you do not need and click the small bin icon on the right of its row.
+4. Read the box that appears and confirm.</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>A box asks Remove saved credentials for &lt;name&gt; (&lt;user&gt;)? and warns You'll need to log in again next time. After confirming, the server disappears from the list and from the Dashboard, and nothing else breaks.</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="n"/>
+      <c r="H63" s="5" t="n"/>
+      <c r="I63" s="5" t="n"/>
+      <c r="J63" s="5" t="n"/>
+    </row>
+    <row r="64" ht="35" customHeight="1">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>9. Tidy Up</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>9.6</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="n"/>
+      <c r="D64" s="5" t="inlineStr">
         <is>
           <t>Remove the app</t>
         </is>
       </c>
-      <c r="E57" s="5" t="inlineStr">
+      <c r="E64" s="5" t="inlineStr">
         <is>
           <t>1. Remove the 45Drives Storage Wizard package the way you normally remove software.</t>
         </is>
       </c>
-      <c r="F57" s="5" t="inlineStr">
+      <c r="F64" s="5" t="inlineStr">
         <is>
           <t>The app is removed with no error messages.</t>
         </is>
       </c>
-      <c r="G57" s="5" t="inlineStr"/>
-      <c r="H57" s="5" t="inlineStr"/>
-      <c r="I57" s="5" t="inlineStr"/>
-      <c r="J57" s="5" t="inlineStr"/>
+      <c r="G64" s="5" t="n"/>
+      <c r="H64" s="5" t="n"/>
+      <c r="I64" s="5" t="n"/>
+      <c r="J64" s="5" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J57"/>
+  <autoFilter ref="A1:J64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2696,7 +2948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A49"/>
+  <dimension ref="A1:A51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="108" customWidth="1" min="1" max="1"/>
@@ -2917,81 +3169,95 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
-    <row r="37">
-      <c r="A37" s="7" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Time. A few tests ask you to close the app, sign out, or leave the computer alone for an hour while a backup runs on its own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>A few words you will see</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Server - the 45Drives machine that stores your files.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Network folder (or share) - the folder on the server that you open from your own computer.</t>
+          <t xml:space="preserve">  Server - the 45Drives machine that stores your files.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Backup - a copy of your files kept on the server, made automatically.</t>
+          <t xml:space="preserve">  Network folder (or share) - the folder on the server that you open from your own computer.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Restore - getting a file back out of a backup.</t>
+          <t xml:space="preserve">  Backup - a copy of your files kept on the server, made automatically.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Restore - getting a file back out of a backup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Dashboard - the main page of the app.</t>
         </is>
       </c>
     </row>
-    <row r="43"/>
     <row r="44">
-      <c r="A44" s="7" t="inlineStr">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Signed out - you have left your user account, but the computer is still switched on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45"/>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
         <is>
           <t>If you get stuck</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t xml:space="preserve">  Write down exactly what you saw, take a screenshot, mark the test FAIL, and carry on to the</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t xml:space="preserve">  next one. Getting stuck is useful information - it means the app was not clear enough.</t>
         </is>
       </c>
     </row>
-    <row r="47"/>
-    <row r="48">
-      <c r="A48" s="7" t="inlineStr">
+    <row r="49"/>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
         <is>
           <t xml:space="preserve">  docs/45Drives_Storage_Wizard_User_Guide.md</t>
         </is>

</xml_diff>